<commit_message>
update data on 17
</commit_message>
<xml_diff>
--- a/2026 1-16 March Number.xlsx
+++ b/2026 1-16 March Number.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://blcppower-my.sharepoint.com/personal/natthaphong_m_blcp_co_th/Documents/BLCP/ATSM 2026/Hot Season/Claude/Fore github/blcp-hotseason-tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{DFC32D05-94C8-4DA2-A566-2308CAAE7D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4454D43-A950-43A2-A929-BBD115D2DF90}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{DFC32D05-94C8-4DA2-A566-2308CAAE7D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4364B755-EA7F-4106-B9B6-BC5639E6A126}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10416" xr2:uid="{84CD358A-30A5-448D-BFC1-D6EF37F91320}"/>
   </bookViews>
@@ -111,6 +111,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -430,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{163996B5-F150-4C6F-BB02-87F4A8F0CBD4}">
-  <dimension ref="A1:D384"/>
+  <dimension ref="A1:D404"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
@@ -5815,6 +5819,286 @@
         <v>38.015998840332031</v>
       </c>
     </row>
+    <row r="385" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A385" s="1">
+        <v>46097.958333333336</v>
+      </c>
+      <c r="B385" s="4">
+        <v>31.105882308062384</v>
+      </c>
+      <c r="C385" s="4">
+        <v>37.384765863418579</v>
+      </c>
+      <c r="D385" s="4">
+        <v>37.995600128173827</v>
+      </c>
+    </row>
+    <row r="386" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A386" s="1">
+        <v>46098</v>
+      </c>
+      <c r="B386" s="4">
+        <v>31.052631679334137</v>
+      </c>
+      <c r="C386" s="4">
+        <v>37.313541730244957</v>
+      </c>
+      <c r="D386" s="4">
+        <v>37.930799102783205</v>
+      </c>
+    </row>
+    <row r="387" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A387" s="1">
+        <v>46098.041666666664</v>
+      </c>
+      <c r="B387" s="4">
+        <v>31.010416587193806</v>
+      </c>
+      <c r="C387" s="4">
+        <v>37.25416666666667</v>
+      </c>
+      <c r="D387" s="4">
+        <v>37.888800048828124</v>
+      </c>
+    </row>
+    <row r="388" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A388" s="1">
+        <v>46098.083333333336</v>
+      </c>
+      <c r="B388" s="4">
+        <v>30.993749976158142</v>
+      </c>
+      <c r="C388" s="4">
+        <v>37.217788696289063</v>
+      </c>
+      <c r="D388" s="4">
+        <v>37.842999776204429</v>
+      </c>
+    </row>
+    <row r="389" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A389" s="1">
+        <v>46098.125</v>
+      </c>
+      <c r="B389" s="4">
+        <v>30.951723953773236</v>
+      </c>
+      <c r="C389" s="4">
+        <v>37.176441779503456</v>
+      </c>
+      <c r="D389" s="4">
+        <v>37.7760009765625</v>
+      </c>
+    </row>
+    <row r="390" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A390" s="1">
+        <v>46098.166666666664</v>
+      </c>
+      <c r="B390" s="4">
+        <v>30.918749862247044</v>
+      </c>
+      <c r="C390" s="4">
+        <v>37.133928298950195</v>
+      </c>
+      <c r="D390" s="4">
+        <v>37.751998901367188</v>
+      </c>
+    </row>
+    <row r="391" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A391" s="1">
+        <v>46098.208333333336</v>
+      </c>
+      <c r="B391" s="4">
+        <v>30.994444246645326</v>
+      </c>
+      <c r="C391" s="4">
+        <v>37.174999745686847</v>
+      </c>
+      <c r="D391" s="4">
+        <v>37.697999954223633</v>
+      </c>
+    </row>
+    <row r="392" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A392" s="1">
+        <v>46098.25</v>
+      </c>
+      <c r="B392" s="4">
+        <v>30.915909073569559</v>
+      </c>
+      <c r="C392" s="4">
+        <v>37.096428734915598</v>
+      </c>
+      <c r="D392" s="4">
+        <v>37.685999870300293</v>
+      </c>
+    </row>
+    <row r="393" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A393" s="1">
+        <v>46098.291666666664</v>
+      </c>
+      <c r="B393" s="4">
+        <v>30.909615443303036</v>
+      </c>
+      <c r="C393" s="4">
+        <v>37.070833418104385</v>
+      </c>
+      <c r="D393" s="4">
+        <v>37.686000061035159</v>
+      </c>
+    </row>
+    <row r="394" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A394" s="1">
+        <v>46098.333333333336</v>
+      </c>
+      <c r="B394" s="4">
+        <v>30.886110305786133</v>
+      </c>
+      <c r="C394" s="4">
+        <v>37.063194274902344</v>
+      </c>
+      <c r="D394" s="4">
+        <v>37.686000823974609</v>
+      </c>
+    </row>
+    <row r="395" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A395" s="1">
+        <v>46098.375</v>
+      </c>
+      <c r="B395" s="4">
+        <v>30.857352425070371</v>
+      </c>
+      <c r="C395" s="4">
+        <v>37.025624847412111</v>
+      </c>
+      <c r="D395" s="4">
+        <v>37.691000620524086</v>
+      </c>
+    </row>
+    <row r="396" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A396" s="1">
+        <v>46098.416666666664</v>
+      </c>
+      <c r="B396" s="4">
+        <v>30.882142748151505</v>
+      </c>
+      <c r="C396" s="4">
+        <v>37.072916666666664</v>
+      </c>
+      <c r="D396" s="4">
+        <v>37.746000289916992</v>
+      </c>
+    </row>
+    <row r="397" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A397" s="1">
+        <v>46098.458333333336</v>
+      </c>
+      <c r="B397" s="4">
+        <v>30.921875</v>
+      </c>
+      <c r="C397" s="4">
+        <v>37.131771087646484</v>
+      </c>
+      <c r="D397" s="4">
+        <v>37.788000106811523</v>
+      </c>
+    </row>
+    <row r="398" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A398" s="1">
+        <v>46098.5</v>
+      </c>
+      <c r="B398" s="4">
+        <v>30.920833428700764</v>
+      </c>
+      <c r="C398" s="4">
+        <v>37.145833333333336</v>
+      </c>
+      <c r="D398" s="4">
+        <v>37.739999771118164</v>
+      </c>
+    </row>
+    <row r="399" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A399" s="1">
+        <v>46098.541666666664</v>
+      </c>
+      <c r="B399" s="4">
+        <v>30.950000127156574</v>
+      </c>
+      <c r="C399" s="4">
+        <v>37.18465874411843</v>
+      </c>
+      <c r="D399" s="4">
+        <v>37.819999694824219</v>
+      </c>
+    </row>
+    <row r="400" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A400" s="1">
+        <v>46098.583333333336</v>
+      </c>
+      <c r="B400" s="4">
+        <v>30.931818181818183</v>
+      </c>
+      <c r="C400" s="4">
+        <v>37.203125</v>
+      </c>
+      <c r="D400" s="4">
+        <v>37.873999277750649</v>
+      </c>
+    </row>
+    <row r="401" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A401" s="1">
+        <v>46098.625</v>
+      </c>
+      <c r="B401" s="4">
+        <v>31.016666730244953</v>
+      </c>
+      <c r="C401" s="4">
+        <v>37.289999898274736</v>
+      </c>
+      <c r="D401" s="4">
+        <v>37.949999237060545</v>
+      </c>
+    </row>
+    <row r="402" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A402" s="1">
+        <v>46098.666666666664</v>
+      </c>
+      <c r="B402" s="4">
+        <v>31.071875333786011</v>
+      </c>
+      <c r="C402" s="4">
+        <v>37.339062690734863</v>
+      </c>
+      <c r="D402" s="4">
+        <v>37.986000061035156</v>
+      </c>
+    </row>
+    <row r="403" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A403" s="1">
+        <v>46098.708333333336</v>
+      </c>
+      <c r="B403" s="4">
+        <v>31.045588100657742</v>
+      </c>
+      <c r="C403" s="4">
+        <v>37.354687213897705</v>
+      </c>
+      <c r="D403" s="4">
+        <v>38.002000172932945</v>
+      </c>
+    </row>
+    <row r="404" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A404" s="1">
+        <v>46098.75</v>
+      </c>
+      <c r="B404" s="4">
+        <v>31</v>
+      </c>
+      <c r="C404" s="4">
+        <v>37.375</v>
+      </c>
+      <c r="D404" s="4">
+        <v>38.058000564575195</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update coal stock and data
</commit_message>
<xml_diff>
--- a/2026 1-16 March Number.xlsx
+++ b/2026 1-16 March Number.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://blcppower-my.sharepoint.com/personal/natthaphong_m_blcp_co_th/Documents/BLCP/ATSM 2026/Hot Season/Claude/Fore github/blcp-hotseason-tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{DFC32D05-94C8-4DA2-A566-2308CAAE7D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8050243-59F3-4BFA-8C4D-2B9F0B7A39EF}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{DFC32D05-94C8-4DA2-A566-2308CAAE7D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A748511-FCB5-4234-8642-8F12AA509F0A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{84CD358A-30A5-448D-BFC1-D6EF37F91320}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10416" xr2:uid="{84CD358A-30A5-448D-BFC1-D6EF37F91320}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -434,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{163996B5-F150-4C6F-BB02-87F4A8F0CBD4}">
-  <dimension ref="A1:D467"/>
+  <dimension ref="A1:D472"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
@@ -6972,13 +6972,83 @@
         <v>46101.375</v>
       </c>
       <c r="B467" s="4">
-        <v>30.740625143051147</v>
+        <v>30.741666793823242</v>
       </c>
       <c r="C467" s="4">
-        <v>37.012500000000003</v>
+        <v>36.990865267240082</v>
       </c>
       <c r="D467" s="4">
-        <v>37.636000315348305</v>
+        <v>37.644999821980797</v>
+      </c>
+    </row>
+    <row r="468" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A468" s="1">
+        <v>46101.416666666664</v>
+      </c>
+      <c r="B468" s="4">
+        <v>30.786841743870784</v>
+      </c>
+      <c r="C468" s="4">
+        <v>37.055682095614344</v>
+      </c>
+      <c r="D468" s="4">
+        <v>37.670999526977539</v>
+      </c>
+    </row>
+    <row r="469" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A469" s="1">
+        <v>46101.458333333336</v>
+      </c>
+      <c r="B469" s="4">
+        <v>30.870833396911621</v>
+      </c>
+      <c r="C469" s="4">
+        <v>37.100567904385656</v>
+      </c>
+      <c r="D469" s="4">
+        <v>37.726799774169919</v>
+      </c>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A470" s="1">
+        <v>46101.5</v>
+      </c>
+      <c r="B470" s="4">
+        <v>30.907692395723782</v>
+      </c>
+      <c r="C470" s="4">
+        <v>37.136363983154297</v>
+      </c>
+      <c r="D470" s="4">
+        <v>37.777713775634766</v>
+      </c>
+    </row>
+    <row r="471" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A471" s="1">
+        <v>46101.541666666664</v>
+      </c>
+      <c r="B471" s="4">
+        <v>30.978125015894573</v>
+      </c>
+      <c r="C471" s="4">
+        <v>37.239062690734862</v>
+      </c>
+      <c r="D471" s="4">
+        <v>37.866000039236887</v>
+      </c>
+    </row>
+    <row r="472" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A472" s="1">
+        <v>46101.583333333336</v>
+      </c>
+      <c r="B472" s="4">
+        <v>31.122222476535374</v>
+      </c>
+      <c r="C472" s="4">
+        <v>37.365104039510094</v>
+      </c>
+      <c r="D472" s="4">
+        <v>37.949332767062714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>